<commit_message>
Melhora o visual do dashboard Excel
Da cara de dashboard (faixa de titulo, fundo de canvas, cartoes brancos
de KPI e rodape em destaque), remove as linhas de grade dos graficos,
limpa os rotulos de dados (so o valor) e reposiciona os graficos para
nao se sobreporem.
</commit_message>
<xml_diff>
--- a/dashboard/dashboard_olist.xlsx
+++ b/dashboard/dashboard_olist.xlsx
@@ -36,7 +36,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4E79"/>
+      <color rgb="00FFFFFF"/>
       <sz val="18"/>
     </font>
     <font>
@@ -66,11 +66,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="001F4E79"/>
-      <sz val="10"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -85,6 +85,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F2F4F5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -119,31 +124,37 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -274,46 +285,12 @@
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
-      <lineChart>
-        <grouping val="standard"/>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'dados_mensal'!F1</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln w="28000">
-              <a:solidFill>
-                <a:srgbClr val="E07B39"/>
-              </a:solidFill>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln>
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
-          <val>
-            <numRef>
-              <f>'dados_mensal'!$F$2:$F$21</f>
-            </numRef>
-          </val>
-        </ser>
-        <axId val="10"/>
-        <axId val="200"/>
-      </lineChart>
       <catAx>
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -325,62 +302,33 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Receita (R$)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
-      <valAx>
-        <axId val="200"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Nota media</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-        <crosses val="max"/>
-      </valAx>
+      <spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
     </plotArea>
-    <legend>
-      <legendPos val="b"/>
-    </legend>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9525">
+      <a:solidFill>
+        <a:srgbClr val="E2E6EA"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -434,7 +382,12 @@
           </val>
         </ser>
         <dLbls>
+          <showLegendKey val="0"/>
           <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
         </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
@@ -445,6 +398,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -456,31 +410,33 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr/>
-              <a:p>
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Nota media (1-5)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
+      <spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
     </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9525">
+      <a:solidFill>
+        <a:srgbClr val="E2E6EA"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -534,7 +490,12 @@
           </val>
         </ser>
         <dLbls>
+          <showLegendKey val="0"/>
           <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
+          <showBubbleSize val="0"/>
         </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
@@ -545,6 +506,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -556,16 +518,33 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
+      <spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
     </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9525">
+      <a:solidFill>
+        <a:srgbClr val="E2E6EA"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -627,6 +606,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -638,16 +618,33 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
-        <majorGridlines/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
       </valAx>
+      <spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </spPr>
     </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln w="9525">
+      <a:solidFill>
+        <a:srgbClr val="E2E6EA"/>
+      </a:solidFill>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -660,7 +657,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="2700000"/>
+    <ext cx="4860000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -682,7 +679,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="2700000"/>
+    <ext cx="4860000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>
@@ -701,10 +698,10 @@
     <from>
       <col>0</col>
       <colOff>0</colOff>
-      <row>24</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="2700000"/>
+    <ext cx="4860000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="3" name="Chart 3"/>
@@ -723,10 +720,10 @@
     <from>
       <col>9</col>
       <colOff>0</colOff>
-      <row>24</row>
+      <row>26</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="2700000"/>
+    <ext cx="4860000" cy="2520000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="4" name="Chart 4"/>
@@ -1033,7 +1030,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R41"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1056,140 +1053,923 @@
     <col width="9" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>OLIST  —  O paradoxo do crescimento: vende mais, mas a entrega ameaca o futuro</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Tech Challenge — Data Analytics | Brazilian E-Commerce Public Dataset by Olist (2017–2018) | Publico: investidores e diretoria</t>
+          <t>OLIST    O paradoxo do crescimento: vende mais, mas a entrega ameaça o futuro</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Tech Challenge · Data Analytics · Olist 2017–2018 · Público: investidores e diretoria</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>RECEITA TOTAL</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="5" t="n"/>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>PEDIDOS</t>
         </is>
       </c>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="E4" s="5" t="n"/>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>TICKET MEDIO</t>
         </is>
       </c>
-      <c r="H4" s="4" t="n"/>
-      <c r="I4" s="4" t="n"/>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="n"/>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="6" t="inlineStr">
         <is>
           <t>TAXA DE RECOMPRA</t>
         </is>
       </c>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="6" t="n"/>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="K4" s="7" t="n"/>
+      <c r="L4" s="7" t="n"/>
+      <c r="M4" s="6" t="inlineStr">
         <is>
           <t>PEDIDOS ATRASADOS</t>
         </is>
       </c>
-      <c r="N4" s="6" t="n"/>
-      <c r="O4" s="6" t="n"/>
+      <c r="N4" s="7" t="n"/>
+      <c r="O4" s="7" t="n"/>
+      <c r="P4" s="8" t="n"/>
+      <c r="Q4" s="8" t="n"/>
+      <c r="R4" s="8" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>R$ 13,5 mi</t>
         </is>
       </c>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="B5" s="10" t="n"/>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t>99.092</t>
         </is>
       </c>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="7" t="inlineStr">
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t>R$ 137,68</t>
         </is>
       </c>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="9" t="inlineStr">
+      <c r="H5" s="10" t="n"/>
+      <c r="I5" s="10" t="n"/>
+      <c r="J5" s="11" t="inlineStr">
         <is>
           <t>3,1%</t>
         </is>
       </c>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="8" t="n"/>
-      <c r="M5" s="9" t="inlineStr">
+      <c r="K5" s="10" t="n"/>
+      <c r="L5" s="10" t="n"/>
+      <c r="M5" s="11" t="inlineStr">
         <is>
           <t>8,1%</t>
         </is>
       </c>
-      <c r="N5" s="8" t="n"/>
-      <c r="O5" s="8" t="n"/>
+      <c r="N5" s="10" t="n"/>
+      <c r="O5" s="10" t="n"/>
+      <c r="P5" s="8" t="n"/>
+      <c r="Q5" s="8" t="n"/>
+      <c r="R5" s="8" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="n"/>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8" t="n"/>
-      <c r="K6" s="8" t="n"/>
-      <c r="L6" s="8" t="n"/>
-      <c r="M6" s="8" t="n"/>
-      <c r="N6" s="8" t="n"/>
-      <c r="O6" s="8" t="n"/>
+      <c r="A6" s="10" t="n"/>
+      <c r="B6" s="10" t="n"/>
+      <c r="C6" s="10" t="n"/>
+      <c r="D6" s="10" t="n"/>
+      <c r="E6" s="10" t="n"/>
+      <c r="F6" s="10" t="n"/>
+      <c r="G6" s="10" t="n"/>
+      <c r="H6" s="10" t="n"/>
+      <c r="I6" s="10" t="n"/>
+      <c r="J6" s="10" t="n"/>
+      <c r="K6" s="10" t="n"/>
+      <c r="L6" s="10" t="n"/>
+      <c r="M6" s="10" t="n"/>
+      <c r="N6" s="10" t="n"/>
+      <c r="O6" s="10" t="n"/>
+      <c r="P6" s="8" t="n"/>
+      <c r="Q6" s="8" t="n"/>
+      <c r="R6" s="8" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
-        <is>
-          <t>Negocio movido a aquisicao (recompra 10x abaixo do mercado ~28%)  →  reputacao e o ativo critico  →  atraso derruba a nota (4,29 → 2,57) e expoe R$ 1,2 mi de receita.</t>
-        </is>
-      </c>
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Negócio movido a aquisição (recompra 10x abaixo do mercado ~28%)  →  reputação é o ativo crítico  →  atraso derruba a nota (4,29 → 2,57) e expõe R$ 1,2 mi de receita.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="8" t="n"/>
+      <c r="K8" s="8" t="n"/>
+      <c r="L8" s="8" t="n"/>
+      <c r="M8" s="8" t="n"/>
+      <c r="N8" s="8" t="n"/>
+      <c r="O8" s="8" t="n"/>
+      <c r="P8" s="8" t="n"/>
+      <c r="Q8" s="8" t="n"/>
+      <c r="R8" s="8" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="8" t="n"/>
+      <c r="C9" s="8" t="n"/>
+      <c r="D9" s="8" t="n"/>
+      <c r="E9" s="8" t="n"/>
+      <c r="F9" s="8" t="n"/>
+      <c r="G9" s="8" t="n"/>
+      <c r="H9" s="8" t="n"/>
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="8" t="n"/>
+      <c r="K9" s="8" t="n"/>
+      <c r="L9" s="8" t="n"/>
+      <c r="M9" s="8" t="n"/>
+      <c r="N9" s="8" t="n"/>
+      <c r="O9" s="8" t="n"/>
+      <c r="P9" s="8" t="n"/>
+      <c r="Q9" s="8" t="n"/>
+      <c r="R9" s="8" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="8" t="n"/>
+      <c r="C10" s="8" t="n"/>
+      <c r="D10" s="8" t="n"/>
+      <c r="E10" s="8" t="n"/>
+      <c r="F10" s="8" t="n"/>
+      <c r="G10" s="8" t="n"/>
+      <c r="H10" s="8" t="n"/>
+      <c r="I10" s="8" t="n"/>
+      <c r="J10" s="8" t="n"/>
+      <c r="K10" s="8" t="n"/>
+      <c r="L10" s="8" t="n"/>
+      <c r="M10" s="8" t="n"/>
+      <c r="N10" s="8" t="n"/>
+      <c r="O10" s="8" t="n"/>
+      <c r="P10" s="8" t="n"/>
+      <c r="Q10" s="8" t="n"/>
+      <c r="R10" s="8" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="8" t="n"/>
+      <c r="C11" s="8" t="n"/>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="8" t="n"/>
+      <c r="F11" s="8" t="n"/>
+      <c r="G11" s="8" t="n"/>
+      <c r="H11" s="8" t="n"/>
+      <c r="I11" s="8" t="n"/>
+      <c r="J11" s="8" t="n"/>
+      <c r="K11" s="8" t="n"/>
+      <c r="L11" s="8" t="n"/>
+      <c r="M11" s="8" t="n"/>
+      <c r="N11" s="8" t="n"/>
+      <c r="O11" s="8" t="n"/>
+      <c r="P11" s="8" t="n"/>
+      <c r="Q11" s="8" t="n"/>
+      <c r="R11" s="8" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="8" t="n"/>
+      <c r="C12" s="8" t="n"/>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="8" t="n"/>
+      <c r="F12" s="8" t="n"/>
+      <c r="G12" s="8" t="n"/>
+      <c r="H12" s="8" t="n"/>
+      <c r="I12" s="8" t="n"/>
+      <c r="J12" s="8" t="n"/>
+      <c r="K12" s="8" t="n"/>
+      <c r="L12" s="8" t="n"/>
+      <c r="M12" s="8" t="n"/>
+      <c r="N12" s="8" t="n"/>
+      <c r="O12" s="8" t="n"/>
+      <c r="P12" s="8" t="n"/>
+      <c r="Q12" s="8" t="n"/>
+      <c r="R12" s="8" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="8" t="n"/>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="8" t="n"/>
+      <c r="F13" s="8" t="n"/>
+      <c r="G13" s="8" t="n"/>
+      <c r="H13" s="8" t="n"/>
+      <c r="I13" s="8" t="n"/>
+      <c r="J13" s="8" t="n"/>
+      <c r="K13" s="8" t="n"/>
+      <c r="L13" s="8" t="n"/>
+      <c r="M13" s="8" t="n"/>
+      <c r="N13" s="8" t="n"/>
+      <c r="O13" s="8" t="n"/>
+      <c r="P13" s="8" t="n"/>
+      <c r="Q13" s="8" t="n"/>
+      <c r="R13" s="8" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="8" t="n"/>
+      <c r="C14" s="8" t="n"/>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="8" t="n"/>
+      <c r="F14" s="8" t="n"/>
+      <c r="G14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
+      <c r="I14" s="8" t="n"/>
+      <c r="J14" s="8" t="n"/>
+      <c r="K14" s="8" t="n"/>
+      <c r="L14" s="8" t="n"/>
+      <c r="M14" s="8" t="n"/>
+      <c r="N14" s="8" t="n"/>
+      <c r="O14" s="8" t="n"/>
+      <c r="P14" s="8" t="n"/>
+      <c r="Q14" s="8" t="n"/>
+      <c r="R14" s="8" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="8" t="n"/>
+      <c r="C15" s="8" t="n"/>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="8" t="n"/>
+      <c r="F15" s="8" t="n"/>
+      <c r="G15" s="8" t="n"/>
+      <c r="H15" s="8" t="n"/>
+      <c r="I15" s="8" t="n"/>
+      <c r="J15" s="8" t="n"/>
+      <c r="K15" s="8" t="n"/>
+      <c r="L15" s="8" t="n"/>
+      <c r="M15" s="8" t="n"/>
+      <c r="N15" s="8" t="n"/>
+      <c r="O15" s="8" t="n"/>
+      <c r="P15" s="8" t="n"/>
+      <c r="Q15" s="8" t="n"/>
+      <c r="R15" s="8" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="8" t="n"/>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
+      <c r="H16" s="8" t="n"/>
+      <c r="I16" s="8" t="n"/>
+      <c r="J16" s="8" t="n"/>
+      <c r="K16" s="8" t="n"/>
+      <c r="L16" s="8" t="n"/>
+      <c r="M16" s="8" t="n"/>
+      <c r="N16" s="8" t="n"/>
+      <c r="O16" s="8" t="n"/>
+      <c r="P16" s="8" t="n"/>
+      <c r="Q16" s="8" t="n"/>
+      <c r="R16" s="8" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+      <c r="H17" s="8" t="n"/>
+      <c r="I17" s="8" t="n"/>
+      <c r="J17" s="8" t="n"/>
+      <c r="K17" s="8" t="n"/>
+      <c r="L17" s="8" t="n"/>
+      <c r="M17" s="8" t="n"/>
+      <c r="N17" s="8" t="n"/>
+      <c r="O17" s="8" t="n"/>
+      <c r="P17" s="8" t="n"/>
+      <c r="Q17" s="8" t="n"/>
+      <c r="R17" s="8" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="8" t="n"/>
+      <c r="H18" s="8" t="n"/>
+      <c r="I18" s="8" t="n"/>
+      <c r="J18" s="8" t="n"/>
+      <c r="K18" s="8" t="n"/>
+      <c r="L18" s="8" t="n"/>
+      <c r="M18" s="8" t="n"/>
+      <c r="N18" s="8" t="n"/>
+      <c r="O18" s="8" t="n"/>
+      <c r="P18" s="8" t="n"/>
+      <c r="Q18" s="8" t="n"/>
+      <c r="R18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="8" t="n"/>
+      <c r="H19" s="8" t="n"/>
+      <c r="I19" s="8" t="n"/>
+      <c r="J19" s="8" t="n"/>
+      <c r="K19" s="8" t="n"/>
+      <c r="L19" s="8" t="n"/>
+      <c r="M19" s="8" t="n"/>
+      <c r="N19" s="8" t="n"/>
+      <c r="O19" s="8" t="n"/>
+      <c r="P19" s="8" t="n"/>
+      <c r="Q19" s="8" t="n"/>
+      <c r="R19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+      <c r="H20" s="8" t="n"/>
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="8" t="n"/>
+      <c r="K20" s="8" t="n"/>
+      <c r="L20" s="8" t="n"/>
+      <c r="M20" s="8" t="n"/>
+      <c r="N20" s="8" t="n"/>
+      <c r="O20" s="8" t="n"/>
+      <c r="P20" s="8" t="n"/>
+      <c r="Q20" s="8" t="n"/>
+      <c r="R20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="8" t="n"/>
+      <c r="H21" s="8" t="n"/>
+      <c r="I21" s="8" t="n"/>
+      <c r="J21" s="8" t="n"/>
+      <c r="K21" s="8" t="n"/>
+      <c r="L21" s="8" t="n"/>
+      <c r="M21" s="8" t="n"/>
+      <c r="N21" s="8" t="n"/>
+      <c r="O21" s="8" t="n"/>
+      <c r="P21" s="8" t="n"/>
+      <c r="Q21" s="8" t="n"/>
+      <c r="R21" s="8" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="8" t="n"/>
+      <c r="C22" s="8" t="n"/>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="8" t="n"/>
+      <c r="F22" s="8" t="n"/>
+      <c r="G22" s="8" t="n"/>
+      <c r="H22" s="8" t="n"/>
+      <c r="I22" s="8" t="n"/>
+      <c r="J22" s="8" t="n"/>
+      <c r="K22" s="8" t="n"/>
+      <c r="L22" s="8" t="n"/>
+      <c r="M22" s="8" t="n"/>
+      <c r="N22" s="8" t="n"/>
+      <c r="O22" s="8" t="n"/>
+      <c r="P22" s="8" t="n"/>
+      <c r="Q22" s="8" t="n"/>
+      <c r="R22" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="8" t="n"/>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="8" t="n"/>
+      <c r="F23" s="8" t="n"/>
+      <c r="G23" s="8" t="n"/>
+      <c r="H23" s="8" t="n"/>
+      <c r="I23" s="8" t="n"/>
+      <c r="J23" s="8" t="n"/>
+      <c r="K23" s="8" t="n"/>
+      <c r="L23" s="8" t="n"/>
+      <c r="M23" s="8" t="n"/>
+      <c r="N23" s="8" t="n"/>
+      <c r="O23" s="8" t="n"/>
+      <c r="P23" s="8" t="n"/>
+      <c r="Q23" s="8" t="n"/>
+      <c r="R23" s="8" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="8" t="n"/>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="8" t="n"/>
+      <c r="F24" s="8" t="n"/>
+      <c r="G24" s="8" t="n"/>
+      <c r="H24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
+      <c r="J24" s="8" t="n"/>
+      <c r="K24" s="8" t="n"/>
+      <c r="L24" s="8" t="n"/>
+      <c r="M24" s="8" t="n"/>
+      <c r="N24" s="8" t="n"/>
+      <c r="O24" s="8" t="n"/>
+      <c r="P24" s="8" t="n"/>
+      <c r="Q24" s="8" t="n"/>
+      <c r="R24" s="8" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="8" t="n"/>
+      <c r="D25" s="8" t="n"/>
+      <c r="E25" s="8" t="n"/>
+      <c r="F25" s="8" t="n"/>
+      <c r="G25" s="8" t="n"/>
+      <c r="H25" s="8" t="n"/>
+      <c r="I25" s="8" t="n"/>
+      <c r="J25" s="8" t="n"/>
+      <c r="K25" s="8" t="n"/>
+      <c r="L25" s="8" t="n"/>
+      <c r="M25" s="8" t="n"/>
+      <c r="N25" s="8" t="n"/>
+      <c r="O25" s="8" t="n"/>
+      <c r="P25" s="8" t="n"/>
+      <c r="Q25" s="8" t="n"/>
+      <c r="R25" s="8" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="8" t="n"/>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="8" t="n"/>
+      <c r="H26" s="8" t="n"/>
+      <c r="I26" s="8" t="n"/>
+      <c r="J26" s="8" t="n"/>
+      <c r="K26" s="8" t="n"/>
+      <c r="L26" s="8" t="n"/>
+      <c r="M26" s="8" t="n"/>
+      <c r="N26" s="8" t="n"/>
+      <c r="O26" s="8" t="n"/>
+      <c r="P26" s="8" t="n"/>
+      <c r="Q26" s="8" t="n"/>
+      <c r="R26" s="8" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="8" t="n"/>
+      <c r="D27" s="8" t="n"/>
+      <c r="E27" s="8" t="n"/>
+      <c r="F27" s="8" t="n"/>
+      <c r="G27" s="8" t="n"/>
+      <c r="H27" s="8" t="n"/>
+      <c r="I27" s="8" t="n"/>
+      <c r="J27" s="8" t="n"/>
+      <c r="K27" s="8" t="n"/>
+      <c r="L27" s="8" t="n"/>
+      <c r="M27" s="8" t="n"/>
+      <c r="N27" s="8" t="n"/>
+      <c r="O27" s="8" t="n"/>
+      <c r="P27" s="8" t="n"/>
+      <c r="Q27" s="8" t="n"/>
+      <c r="R27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="8" t="n"/>
+      <c r="C28" s="8" t="n"/>
+      <c r="D28" s="8" t="n"/>
+      <c r="E28" s="8" t="n"/>
+      <c r="F28" s="8" t="n"/>
+      <c r="G28" s="8" t="n"/>
+      <c r="H28" s="8" t="n"/>
+      <c r="I28" s="8" t="n"/>
+      <c r="J28" s="8" t="n"/>
+      <c r="K28" s="8" t="n"/>
+      <c r="L28" s="8" t="n"/>
+      <c r="M28" s="8" t="n"/>
+      <c r="N28" s="8" t="n"/>
+      <c r="O28" s="8" t="n"/>
+      <c r="P28" s="8" t="n"/>
+      <c r="Q28" s="8" t="n"/>
+      <c r="R28" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="8" t="n"/>
+      <c r="C29" s="8" t="n"/>
+      <c r="D29" s="8" t="n"/>
+      <c r="E29" s="8" t="n"/>
+      <c r="F29" s="8" t="n"/>
+      <c r="G29" s="8" t="n"/>
+      <c r="H29" s="8" t="n"/>
+      <c r="I29" s="8" t="n"/>
+      <c r="J29" s="8" t="n"/>
+      <c r="K29" s="8" t="n"/>
+      <c r="L29" s="8" t="n"/>
+      <c r="M29" s="8" t="n"/>
+      <c r="N29" s="8" t="n"/>
+      <c r="O29" s="8" t="n"/>
+      <c r="P29" s="8" t="n"/>
+      <c r="Q29" s="8" t="n"/>
+      <c r="R29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="8" t="n"/>
+      <c r="C30" s="8" t="n"/>
+      <c r="D30" s="8" t="n"/>
+      <c r="E30" s="8" t="n"/>
+      <c r="F30" s="8" t="n"/>
+      <c r="G30" s="8" t="n"/>
+      <c r="H30" s="8" t="n"/>
+      <c r="I30" s="8" t="n"/>
+      <c r="J30" s="8" t="n"/>
+      <c r="K30" s="8" t="n"/>
+      <c r="L30" s="8" t="n"/>
+      <c r="M30" s="8" t="n"/>
+      <c r="N30" s="8" t="n"/>
+      <c r="O30" s="8" t="n"/>
+      <c r="P30" s="8" t="n"/>
+      <c r="Q30" s="8" t="n"/>
+      <c r="R30" s="8" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="8" t="n"/>
+      <c r="C31" s="8" t="n"/>
+      <c r="D31" s="8" t="n"/>
+      <c r="E31" s="8" t="n"/>
+      <c r="F31" s="8" t="n"/>
+      <c r="G31" s="8" t="n"/>
+      <c r="H31" s="8" t="n"/>
+      <c r="I31" s="8" t="n"/>
+      <c r="J31" s="8" t="n"/>
+      <c r="K31" s="8" t="n"/>
+      <c r="L31" s="8" t="n"/>
+      <c r="M31" s="8" t="n"/>
+      <c r="N31" s="8" t="n"/>
+      <c r="O31" s="8" t="n"/>
+      <c r="P31" s="8" t="n"/>
+      <c r="Q31" s="8" t="n"/>
+      <c r="R31" s="8" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="8" t="n"/>
+      <c r="C32" s="8" t="n"/>
+      <c r="D32" s="8" t="n"/>
+      <c r="E32" s="8" t="n"/>
+      <c r="F32" s="8" t="n"/>
+      <c r="G32" s="8" t="n"/>
+      <c r="H32" s="8" t="n"/>
+      <c r="I32" s="8" t="n"/>
+      <c r="J32" s="8" t="n"/>
+      <c r="K32" s="8" t="n"/>
+      <c r="L32" s="8" t="n"/>
+      <c r="M32" s="8" t="n"/>
+      <c r="N32" s="8" t="n"/>
+      <c r="O32" s="8" t="n"/>
+      <c r="P32" s="8" t="n"/>
+      <c r="Q32" s="8" t="n"/>
+      <c r="R32" s="8" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
+      <c r="D33" s="8" t="n"/>
+      <c r="E33" s="8" t="n"/>
+      <c r="F33" s="8" t="n"/>
+      <c r="G33" s="8" t="n"/>
+      <c r="H33" s="8" t="n"/>
+      <c r="I33" s="8" t="n"/>
+      <c r="J33" s="8" t="n"/>
+      <c r="K33" s="8" t="n"/>
+      <c r="L33" s="8" t="n"/>
+      <c r="M33" s="8" t="n"/>
+      <c r="N33" s="8" t="n"/>
+      <c r="O33" s="8" t="n"/>
+      <c r="P33" s="8" t="n"/>
+      <c r="Q33" s="8" t="n"/>
+      <c r="R33" s="8" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="8" t="n"/>
+      <c r="C34" s="8" t="n"/>
+      <c r="D34" s="8" t="n"/>
+      <c r="E34" s="8" t="n"/>
+      <c r="F34" s="8" t="n"/>
+      <c r="G34" s="8" t="n"/>
+      <c r="H34" s="8" t="n"/>
+      <c r="I34" s="8" t="n"/>
+      <c r="J34" s="8" t="n"/>
+      <c r="K34" s="8" t="n"/>
+      <c r="L34" s="8" t="n"/>
+      <c r="M34" s="8" t="n"/>
+      <c r="N34" s="8" t="n"/>
+      <c r="O34" s="8" t="n"/>
+      <c r="P34" s="8" t="n"/>
+      <c r="Q34" s="8" t="n"/>
+      <c r="R34" s="8" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="8" t="n"/>
+      <c r="C35" s="8" t="n"/>
+      <c r="D35" s="8" t="n"/>
+      <c r="E35" s="8" t="n"/>
+      <c r="F35" s="8" t="n"/>
+      <c r="G35" s="8" t="n"/>
+      <c r="H35" s="8" t="n"/>
+      <c r="I35" s="8" t="n"/>
+      <c r="J35" s="8" t="n"/>
+      <c r="K35" s="8" t="n"/>
+      <c r="L35" s="8" t="n"/>
+      <c r="M35" s="8" t="n"/>
+      <c r="N35" s="8" t="n"/>
+      <c r="O35" s="8" t="n"/>
+      <c r="P35" s="8" t="n"/>
+      <c r="Q35" s="8" t="n"/>
+      <c r="R35" s="8" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n"/>
+      <c r="B36" s="8" t="n"/>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="8" t="n"/>
+      <c r="H36" s="8" t="n"/>
+      <c r="I36" s="8" t="n"/>
+      <c r="J36" s="8" t="n"/>
+      <c r="K36" s="8" t="n"/>
+      <c r="L36" s="8" t="n"/>
+      <c r="M36" s="8" t="n"/>
+      <c r="N36" s="8" t="n"/>
+      <c r="O36" s="8" t="n"/>
+      <c r="P36" s="8" t="n"/>
+      <c r="Q36" s="8" t="n"/>
+      <c r="R36" s="8" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="8" t="n"/>
+      <c r="C37" s="8" t="n"/>
+      <c r="D37" s="8" t="n"/>
+      <c r="E37" s="8" t="n"/>
+      <c r="F37" s="8" t="n"/>
+      <c r="G37" s="8" t="n"/>
+      <c r="H37" s="8" t="n"/>
+      <c r="I37" s="8" t="n"/>
+      <c r="J37" s="8" t="n"/>
+      <c r="K37" s="8" t="n"/>
+      <c r="L37" s="8" t="n"/>
+      <c r="M37" s="8" t="n"/>
+      <c r="N37" s="8" t="n"/>
+      <c r="O37" s="8" t="n"/>
+      <c r="P37" s="8" t="n"/>
+      <c r="Q37" s="8" t="n"/>
+      <c r="R37" s="8" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n"/>
+      <c r="B38" s="8" t="n"/>
+      <c r="C38" s="8" t="n"/>
+      <c r="D38" s="8" t="n"/>
+      <c r="E38" s="8" t="n"/>
+      <c r="F38" s="8" t="n"/>
+      <c r="G38" s="8" t="n"/>
+      <c r="H38" s="8" t="n"/>
+      <c r="I38" s="8" t="n"/>
+      <c r="J38" s="8" t="n"/>
+      <c r="K38" s="8" t="n"/>
+      <c r="L38" s="8" t="n"/>
+      <c r="M38" s="8" t="n"/>
+      <c r="N38" s="8" t="n"/>
+      <c r="O38" s="8" t="n"/>
+      <c r="P38" s="8" t="n"/>
+      <c r="Q38" s="8" t="n"/>
+      <c r="R38" s="8" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n"/>
+      <c r="B39" s="8" t="n"/>
+      <c r="C39" s="8" t="n"/>
+      <c r="D39" s="8" t="n"/>
+      <c r="E39" s="8" t="n"/>
+      <c r="F39" s="8" t="n"/>
+      <c r="G39" s="8" t="n"/>
+      <c r="H39" s="8" t="n"/>
+      <c r="I39" s="8" t="n"/>
+      <c r="J39" s="8" t="n"/>
+      <c r="K39" s="8" t="n"/>
+      <c r="L39" s="8" t="n"/>
+      <c r="M39" s="8" t="n"/>
+      <c r="N39" s="8" t="n"/>
+      <c r="O39" s="8" t="n"/>
+      <c r="P39" s="8" t="n"/>
+      <c r="Q39" s="8" t="n"/>
+      <c r="R39" s="8" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n"/>
+      <c r="B40" s="8" t="n"/>
+      <c r="C40" s="8" t="n"/>
+      <c r="D40" s="8" t="n"/>
+      <c r="E40" s="8" t="n"/>
+      <c r="F40" s="8" t="n"/>
+      <c r="G40" s="8" t="n"/>
+      <c r="H40" s="8" t="n"/>
+      <c r="I40" s="8" t="n"/>
+      <c r="J40" s="8" t="n"/>
+      <c r="K40" s="8" t="n"/>
+      <c r="L40" s="8" t="n"/>
+      <c r="M40" s="8" t="n"/>
+      <c r="N40" s="8" t="n"/>
+      <c r="O40" s="8" t="n"/>
+      <c r="P40" s="8" t="n"/>
+      <c r="Q40" s="8" t="n"/>
+      <c r="R40" s="8" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="inlineStr">
-        <is>
-          <t>Logistica nao e custo — e a alavanca que protege o crescimento. Reduzir atrasos em 50% protege ~R$ 579 mil e evita ~1.755 detratores.</t>
-        </is>
-      </c>
+      <c r="A41" s="8" t="n"/>
+      <c r="B41" s="8" t="n"/>
+      <c r="C41" s="8" t="n"/>
+      <c r="D41" s="8" t="n"/>
+      <c r="E41" s="8" t="n"/>
+      <c r="F41" s="8" t="n"/>
+      <c r="G41" s="8" t="n"/>
+      <c r="H41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
+      <c r="J41" s="8" t="n"/>
+      <c r="K41" s="8" t="n"/>
+      <c r="L41" s="8" t="n"/>
+      <c r="M41" s="8" t="n"/>
+      <c r="N41" s="8" t="n"/>
+      <c r="O41" s="8" t="n"/>
+      <c r="P41" s="8" t="n"/>
+      <c r="Q41" s="8" t="n"/>
+      <c r="R41" s="8" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="8" t="n"/>
+      <c r="F42" s="8" t="n"/>
+      <c r="G42" s="8" t="n"/>
+      <c r="H42" s="8" t="n"/>
+      <c r="I42" s="8" t="n"/>
+      <c r="J42" s="8" t="n"/>
+      <c r="K42" s="8" t="n"/>
+      <c r="L42" s="8" t="n"/>
+      <c r="M42" s="8" t="n"/>
+      <c r="N42" s="8" t="n"/>
+      <c r="O42" s="8" t="n"/>
+      <c r="P42" s="8" t="n"/>
+      <c r="Q42" s="8" t="n"/>
+      <c r="R42" s="8" t="n"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
+        <is>
+          <t>Logística não é custo: é a alavanca que protege o crescimento.   Reduzir atrasos em 50% protege ~R$ 579 mil e evita ~1.755 detratores.</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="n"/>
+      <c r="C43" s="2" t="n"/>
+      <c r="D43" s="2" t="n"/>
+      <c r="E43" s="2" t="n"/>
+      <c r="F43" s="2" t="n"/>
+      <c r="G43" s="2" t="n"/>
+      <c r="H43" s="2" t="n"/>
+      <c r="I43" s="2" t="n"/>
+      <c r="J43" s="2" t="n"/>
+      <c r="K43" s="2" t="n"/>
+      <c r="L43" s="2" t="n"/>
+      <c r="M43" s="2" t="n"/>
+      <c r="N43" s="2" t="n"/>
+      <c r="O43" s="2" t="n"/>
+      <c r="P43" s="2" t="n"/>
+      <c r="Q43" s="2" t="n"/>
+      <c r="R43" s="2" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n"/>
+      <c r="B44" s="8" t="n"/>
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="8" t="n"/>
+      <c r="E44" s="8" t="n"/>
+      <c r="F44" s="8" t="n"/>
+      <c r="G44" s="8" t="n"/>
+      <c r="H44" s="8" t="n"/>
+      <c r="I44" s="8" t="n"/>
+      <c r="J44" s="8" t="n"/>
+      <c r="K44" s="8" t="n"/>
+      <c r="L44" s="8" t="n"/>
+      <c r="M44" s="8" t="n"/>
+      <c r="N44" s="8" t="n"/>
+      <c r="O44" s="8" t="n"/>
+      <c r="P44" s="8" t="n"/>
+      <c r="Q44" s="8" t="n"/>
+      <c r="R44" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A3:R3"/>
     <mergeCell ref="A7:R7"/>
-    <mergeCell ref="A41:R41"/>
-    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A43:R43"/>
+    <mergeCell ref="D5:F6"/>
     <mergeCell ref="A5:C6"/>
-    <mergeCell ref="D5:F6"/>
+    <mergeCell ref="G5:I6"/>
     <mergeCell ref="D4:F4"/>
-    <mergeCell ref="G5:I6"/>
     <mergeCell ref="M4:O4"/>
     <mergeCell ref="M5:O6"/>
     <mergeCell ref="J5:L6"/>
     <mergeCell ref="G4:I4"/>
-    <mergeCell ref="A1:R1"/>
     <mergeCell ref="J4:L4"/>
+    <mergeCell ref="A1:R2"/>
     <mergeCell ref="A4:C4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1207,32 +1987,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>ano_mes</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>pedidos</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>receita</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>ticket_medio</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>pct_atraso</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>nota_media</t>
         </is>
@@ -1693,17 +2473,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>faixa_atraso</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>nota_media</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>pedidos</t>
         </is>
@@ -1802,22 +2582,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>cenario</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>reducao_pct</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>receita_protegida</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>detratores_evitados</t>
         </is>
@@ -1886,27 +2666,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>pedidos</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>receita</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>ticket_medio</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>nota_media</t>
         </is>
@@ -2079,32 +2859,32 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="inlineStr">
+      <c r="A1" s="14" t="inlineStr">
         <is>
           <t>uf</t>
         </is>
       </c>
-      <c r="B1" s="12" t="inlineStr">
+      <c r="B1" s="14" t="inlineStr">
         <is>
           <t>pedidos</t>
         </is>
       </c>
-      <c r="C1" s="12" t="inlineStr">
+      <c r="C1" s="14" t="inlineStr">
         <is>
           <t>receita</t>
         </is>
       </c>
-      <c r="D1" s="12" t="inlineStr">
+      <c r="D1" s="14" t="inlineStr">
         <is>
           <t>prazo_medio_dias</t>
         </is>
       </c>
-      <c r="E1" s="12" t="inlineStr">
+      <c r="E1" s="14" t="inlineStr">
         <is>
           <t>pct_atraso</t>
         </is>
       </c>
-      <c r="F1" s="12" t="inlineStr">
+      <c r="F1" s="14" t="inlineStr">
         <is>
           <t>nota_media</t>
         </is>

</xml_diff>